<commit_message>
Shiny app update and moderator meta analysis
</commit_message>
<xml_diff>
--- a/output/long_format_with_newcol.xlsx
+++ b/output/long_format_with_newcol.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\smprchan\Documents\R Programming\agewell_tudo\AgeYouth\output\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D7B111D-43A4-4543-A5C4-05A44CC065B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12180"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -18,9 +24,10 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -2120,14 +2127,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="21">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -2135,353 +2136,16 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="33">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -2489,338 +2153,165 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
       <border>
@@ -2831,7 +2322,7 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="0"/>
       </font>
       <fill>
@@ -2859,154 +2350,40 @@
           <color theme="4"/>
         </bottom>
         <horizontal style="thin">
-          <color theme="4" tint="0.399975585192419"/>
+          <color theme="4" tint="0.39994506668294322"/>
         </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
       </border>
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
     <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+      <tableStyleElement type="wholeTable" dxfId="16"/>
+      <tableStyleElement type="headerRow" dxfId="15"/>
+      <tableStyleElement type="totalRow" dxfId="14"/>
+      <tableStyleElement type="firstColumn" dxfId="13"/>
+      <tableStyleElement type="lastColumn" dxfId="12"/>
+      <tableStyleElement type="firstRowStripe" dxfId="11"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="10"/>
     </tableStyle>
     <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="totalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
-      <tableStyleElement type="pageFieldValues" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="9"/>
+      <tableStyleElement type="totalRow" dxfId="8"/>
+      <tableStyleElement type="firstRowStripe" dxfId="7"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="6"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="5"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="4"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="3"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="2"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="1"/>
+      <tableStyleElement type="pageFieldValues" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -3285,14 +2662,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V464"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:22">
       <c r="A1" t="s">
@@ -3486,7 +2863,7 @@
         <v>1.73</v>
       </c>
       <c r="S3">
-        <v>9.7</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="T3">
         <v>1.71</v>
@@ -3616,7 +2993,7 @@
         <v>48</v>
       </c>
       <c r="Q5">
-        <v>9.46</v>
+        <v>9.4600000000000009</v>
       </c>
       <c r="R5">
         <v>1.9</v>
@@ -3891,13 +3268,13 @@
         <v>2.25</v>
       </c>
       <c r="R9">
-        <v>0.55</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="S9">
         <v>2.17</v>
       </c>
       <c r="T9">
-        <v>0.55</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="U9">
         <v>0.02</v>
@@ -4030,7 +3407,7 @@
         <v>0.76</v>
       </c>
       <c r="S11">
-        <v>4.69</v>
+        <v>4.6900000000000004</v>
       </c>
       <c r="T11">
         <v>0.87</v>
@@ -4092,7 +3469,7 @@
         <v>33</v>
       </c>
       <c r="Q12">
-        <v>4.69</v>
+        <v>4.6900000000000004</v>
       </c>
       <c r="R12">
         <v>0.87</v>
@@ -4166,7 +3543,7 @@
         <v>0.88</v>
       </c>
       <c r="S13">
-        <v>4.48</v>
+        <v>4.4800000000000004</v>
       </c>
       <c r="T13">
         <v>0.88</v>
@@ -4784,7 +4161,7 @@
         <v>0.68</v>
       </c>
       <c r="U22">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="V22">
         <v>0.5</v>
@@ -4976,7 +4353,7 @@
         <v>56</v>
       </c>
       <c r="Q25">
-        <v>8.45</v>
+        <v>8.4499999999999993</v>
       </c>
       <c r="R25">
         <v>8.06</v>
@@ -5041,7 +4418,7 @@
         <v>6.06</v>
       </c>
       <c r="R26">
-        <v>1.16</v>
+        <v>1.1599999999999999</v>
       </c>
       <c r="S26">
         <v>5.64</v>
@@ -5109,7 +4486,7 @@
         <v>5.4</v>
       </c>
       <c r="R27">
-        <v>1.13</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="S27">
         <v>5.58</v>
@@ -5118,7 +4495,7 @@
         <v>1.05</v>
       </c>
       <c r="U27">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="V27">
         <v>1</v>
@@ -5180,7 +4557,7 @@
         <v>1.24</v>
       </c>
       <c r="S28">
-        <v>4.98</v>
+        <v>4.9800000000000004</v>
       </c>
       <c r="T28">
         <v>1.2</v>
@@ -5254,7 +4631,7 @@
         <v>6.45</v>
       </c>
       <c r="U29">
-        <v>0.55</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="V29">
         <v>1</v>
@@ -5310,7 +4687,7 @@
         <v>118</v>
       </c>
       <c r="Q30">
-        <v>32.2</v>
+        <v>32.200000000000003</v>
       </c>
       <c r="R30">
         <v>5.5</v>
@@ -5650,7 +5027,7 @@
         <v>135</v>
       </c>
       <c r="Q35">
-        <v>16.4</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="R35">
         <v>3.2</v>
@@ -5792,7 +5169,7 @@
         <v>3.3</v>
       </c>
       <c r="S37">
-        <v>17.4</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="T37">
         <v>3.5</v>
@@ -6064,7 +5441,7 @@
         <v>1.39</v>
       </c>
       <c r="S41">
-        <v>5.02</v>
+        <v>5.0199999999999996</v>
       </c>
       <c r="T41">
         <v>1.3</v>
@@ -6206,7 +5583,7 @@
         <v>0.79</v>
       </c>
       <c r="U43">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="V43">
         <v>0.5</v>
@@ -6330,7 +5707,7 @@
         <v>62</v>
       </c>
       <c r="Q45">
-        <v>2.55</v>
+        <v>2.5499999999999998</v>
       </c>
       <c r="R45">
         <v>0.79</v>
@@ -6605,10 +5982,10 @@
         <v>18.8</v>
       </c>
       <c r="R49">
-        <v>4.48</v>
+        <v>4.4800000000000004</v>
       </c>
       <c r="S49">
-        <v>18.35</v>
+        <v>18.350000000000001</v>
       </c>
       <c r="T49">
         <v>4.41</v>
@@ -6676,7 +6053,7 @@
         <v>0.65</v>
       </c>
       <c r="S50">
-        <v>4.61</v>
+        <v>4.6100000000000003</v>
       </c>
       <c r="T50">
         <v>0.7</v>
@@ -6800,7 +6177,7 @@
         <v>85</v>
       </c>
       <c r="Q52">
-        <v>72.6</v>
+        <v>72.599999999999994</v>
       </c>
       <c r="R52">
         <v>20.2</v>
@@ -6874,7 +6251,7 @@
         <v>19.3</v>
       </c>
       <c r="S53">
-        <v>72.6</v>
+        <v>72.599999999999994</v>
       </c>
       <c r="T53">
         <v>23</v>
@@ -6936,13 +6313,13 @@
         <v>85</v>
       </c>
       <c r="Q54">
-        <v>72.6</v>
+        <v>72.599999999999994</v>
       </c>
       <c r="R54">
         <v>23</v>
       </c>
       <c r="S54">
-        <v>72.9</v>
+        <v>72.900000000000006</v>
       </c>
       <c r="T54">
         <v>20.6</v>
@@ -7149,7 +6526,7 @@
         <v>1.71</v>
       </c>
       <c r="T57">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="U57">
         <v>9999</v>
@@ -7211,13 +6588,13 @@
         <v>1.71</v>
       </c>
       <c r="R58">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="S58">
         <v>1.67</v>
       </c>
       <c r="T58">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="U58">
         <v>9999</v>
@@ -7486,7 +6863,7 @@
         <v>3.32</v>
       </c>
       <c r="S62">
-        <v>9.13</v>
+        <v>9.1300000000000008</v>
       </c>
       <c r="T62">
         <v>3.53</v>
@@ -7548,7 +6925,7 @@
         <v>187</v>
       </c>
       <c r="Q63">
-        <v>9.13</v>
+        <v>9.1300000000000008</v>
       </c>
       <c r="R63">
         <v>3.53</v>
@@ -7820,7 +7197,7 @@
         <v>195</v>
       </c>
       <c r="Q67">
-        <v>34.45</v>
+        <v>34.450000000000003</v>
       </c>
       <c r="R67">
         <v>6.37</v>
@@ -7968,7 +7345,7 @@
         <v>0.66</v>
       </c>
       <c r="U69">
-        <v>0.55</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="V69">
         <v>1</v>
@@ -8163,7 +7540,7 @@
         <v>3.16</v>
       </c>
       <c r="R72">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="S72">
         <v>3.17</v>
@@ -8571,7 +7948,7 @@
         <v>3.18</v>
       </c>
       <c r="R78">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="S78">
         <v>3.16</v>
@@ -8846,7 +8223,7 @@
         <v>1.18</v>
       </c>
       <c r="S82">
-        <v>4.02</v>
+        <v>4.0199999999999996</v>
       </c>
       <c r="T82">
         <v>1.17</v>
@@ -8917,7 +8294,7 @@
         <v>5.39</v>
       </c>
       <c r="T83">
-        <v>1.15</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="U83">
         <v>0.32</v>
@@ -9665,7 +9042,7 @@
         <v>3.22</v>
       </c>
       <c r="T94">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="U94">
         <v>9999</v>
@@ -9866,7 +9243,7 @@
         <v>1.23</v>
       </c>
       <c r="S97">
-        <v>4.89</v>
+        <v>4.8899999999999997</v>
       </c>
       <c r="T97">
         <v>1.32</v>
@@ -9928,16 +9305,16 @@
         <v>66</v>
       </c>
       <c r="Q98">
-        <v>4.48</v>
+        <v>4.4800000000000004</v>
       </c>
       <c r="R98">
         <v>0.52</v>
       </c>
       <c r="S98">
-        <v>4.39</v>
+        <v>4.3899999999999997</v>
       </c>
       <c r="T98">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="U98">
         <v>9999</v>
@@ -9990,13 +9367,13 @@
         <v>75</v>
       </c>
       <c r="Q99">
-        <v>2.55</v>
+        <v>2.5499999999999998</v>
       </c>
       <c r="R99">
         <v>0.8</v>
       </c>
       <c r="S99">
-        <v>2.53</v>
+        <v>2.5299999999999998</v>
       </c>
       <c r="T99">
         <v>0.74</v>
@@ -10052,13 +9429,13 @@
         <v>75</v>
       </c>
       <c r="Q100">
-        <v>2.53</v>
+        <v>2.5299999999999998</v>
       </c>
       <c r="R100">
         <v>0.74</v>
       </c>
       <c r="S100">
-        <v>2.49</v>
+        <v>2.4900000000000002</v>
       </c>
       <c r="T100">
         <v>0.74</v>
@@ -10114,13 +9491,13 @@
         <v>75</v>
       </c>
       <c r="Q101">
-        <v>2.49</v>
+        <v>2.4900000000000002</v>
       </c>
       <c r="R101">
         <v>0.74</v>
       </c>
       <c r="S101">
-        <v>2.47</v>
+        <v>2.4700000000000002</v>
       </c>
       <c r="T101">
         <v>0.74</v>
@@ -10176,7 +9553,7 @@
         <v>75</v>
       </c>
       <c r="Q102">
-        <v>2.47</v>
+        <v>2.4700000000000002</v>
       </c>
       <c r="R102">
         <v>0.74</v>
@@ -10392,7 +9769,7 @@
         <v>1.25</v>
       </c>
       <c r="U105">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="V105">
         <v>1</v>
@@ -10460,7 +9837,7 @@
         <v>1.27</v>
       </c>
       <c r="U106">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="V106">
         <v>1</v>
@@ -10525,7 +9902,7 @@
         <v>2.88</v>
       </c>
       <c r="T107">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="U107">
         <v>9999</v>
@@ -10587,13 +9964,13 @@
         <v>2.88</v>
       </c>
       <c r="R108">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="S108">
         <v>2.9</v>
       </c>
       <c r="T108">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="U108">
         <v>9999</v>
@@ -10655,7 +10032,7 @@
         <v>3.13</v>
       </c>
       <c r="R109">
-        <v>0.55</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="S109">
         <v>3.07</v>
@@ -11134,7 +10511,7 @@
         <v>1.43</v>
       </c>
       <c r="S116">
-        <v>8.13</v>
+        <v>8.1300000000000008</v>
       </c>
       <c r="T116">
         <v>1.66</v>
@@ -11199,13 +10576,13 @@
         <v>2.11</v>
       </c>
       <c r="R117">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="S117">
         <v>2.09</v>
       </c>
       <c r="T117">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="U117">
         <v>9999</v>
@@ -11267,7 +10644,7 @@
         <v>2.09</v>
       </c>
       <c r="R118">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="S118">
         <v>2.04</v>
@@ -11672,7 +11049,7 @@
         <v>48</v>
       </c>
       <c r="Q124">
-        <v>4.11</v>
+        <v>4.1100000000000003</v>
       </c>
       <c r="R124">
         <v>0.65</v>
@@ -11743,13 +11120,13 @@
         <v>4.76</v>
       </c>
       <c r="R125">
-        <v>1.11</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="S125">
         <v>4.71</v>
       </c>
       <c r="T125">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="U125">
         <v>9999</v>
@@ -11882,7 +11259,7 @@
         <v>3.85</v>
       </c>
       <c r="S127">
-        <v>16.24</v>
+        <v>16.239999999999998</v>
       </c>
       <c r="T127">
         <v>3.66</v>
@@ -12009,7 +11386,7 @@
         <v>5.37</v>
       </c>
       <c r="R129">
-        <v>2.2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="S129">
         <v>6.68</v>
@@ -12352,7 +11729,7 @@
         <v>0.7</v>
       </c>
       <c r="U134">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="V134">
         <v>0.33</v>
@@ -12414,13 +11791,13 @@
         <v>0.73</v>
       </c>
       <c r="S135">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="T135">
         <v>0.76</v>
       </c>
       <c r="U135">
-        <v>0.55</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="V135">
         <v>0.42</v>
@@ -12476,13 +11853,13 @@
         <v>111</v>
       </c>
       <c r="Q136">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="R136">
         <v>0.76</v>
       </c>
       <c r="S136">
-        <v>2.32</v>
+        <v>2.3199999999999998</v>
       </c>
       <c r="T136">
         <v>0.74</v>
@@ -12559,7 +11936,7 @@
         <v>0.46</v>
       </c>
       <c r="V137">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
     </row>
     <row r="138" spans="1:22">
@@ -12748,7 +12125,7 @@
         <v>157</v>
       </c>
       <c r="Q140">
-        <v>4.81</v>
+        <v>4.8099999999999996</v>
       </c>
       <c r="R140">
         <v>1.23</v>
@@ -12896,7 +12273,7 @@
         <v>3.01</v>
       </c>
       <c r="U142">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="V142">
         <v>0.5</v>
@@ -13032,7 +12409,7 @@
         <v>1.28</v>
       </c>
       <c r="U144">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="V144">
         <v>0.5</v>
@@ -13100,7 +12477,7 @@
         <v>1.29</v>
       </c>
       <c r="U145">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="V145">
         <v>0.5</v>
@@ -13295,13 +12672,13 @@
         <v>4.82</v>
       </c>
       <c r="R148">
-        <v>1.12</v>
+        <v>1.1200000000000001</v>
       </c>
       <c r="S148">
-        <v>4.81</v>
+        <v>4.8099999999999996</v>
       </c>
       <c r="T148">
-        <v>1.13</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="U148">
         <v>9999</v>
@@ -13366,7 +12743,7 @@
         <v>0.76</v>
       </c>
       <c r="S149">
-        <v>4.69</v>
+        <v>4.6900000000000004</v>
       </c>
       <c r="T149">
         <v>0.87</v>
@@ -13428,7 +12805,7 @@
         <v>187</v>
       </c>
       <c r="Q150">
-        <v>4.69</v>
+        <v>4.6900000000000004</v>
       </c>
       <c r="R150">
         <v>0.87</v>
@@ -13502,13 +12879,13 @@
         <v>0.88</v>
       </c>
       <c r="S151">
-        <v>4.48</v>
+        <v>4.4800000000000004</v>
       </c>
       <c r="T151">
         <v>0.88</v>
       </c>
       <c r="U151">
-        <v>0.55</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="V151">
         <v>1</v>
@@ -14099,13 +13476,13 @@
         <v>3.91</v>
       </c>
       <c r="R160">
-        <v>1.14</v>
+        <v>1.1399999999999999</v>
       </c>
       <c r="S160">
-        <v>4.06</v>
+        <v>4.0599999999999996</v>
       </c>
       <c r="T160">
-        <v>1.13</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="U160">
         <v>0.61</v>
@@ -14164,16 +13541,16 @@
         <v>111</v>
       </c>
       <c r="Q161">
-        <v>4.06</v>
+        <v>4.0599999999999996</v>
       </c>
       <c r="R161">
-        <v>1.13</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="S161">
-        <v>4.19</v>
+        <v>4.1900000000000004</v>
       </c>
       <c r="T161">
-        <v>1.14</v>
+        <v>1.1399999999999999</v>
       </c>
       <c r="U161">
         <v>0.63</v>
@@ -14232,13 +13609,13 @@
         <v>111</v>
       </c>
       <c r="Q162">
-        <v>4.19</v>
+        <v>4.1900000000000004</v>
       </c>
       <c r="R162">
-        <v>1.14</v>
+        <v>1.1399999999999999</v>
       </c>
       <c r="S162">
-        <v>4.19</v>
+        <v>4.1900000000000004</v>
       </c>
       <c r="T162">
         <v>1.03</v>
@@ -14303,13 +13680,13 @@
         <v>3.83</v>
       </c>
       <c r="R163">
-        <v>1.12</v>
+        <v>1.1200000000000001</v>
       </c>
       <c r="S163">
         <v>3.91</v>
       </c>
       <c r="T163">
-        <v>1.14</v>
+        <v>1.1399999999999999</v>
       </c>
       <c r="U163">
         <v>0.64</v>
@@ -14371,13 +13748,13 @@
         <v>3.91</v>
       </c>
       <c r="R164">
-        <v>1.14</v>
+        <v>1.1399999999999999</v>
       </c>
       <c r="S164">
         <v>4.03</v>
       </c>
       <c r="T164">
-        <v>1.13</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="U164">
         <v>0.61</v>
@@ -14439,7 +13816,7 @@
         <v>4.03</v>
       </c>
       <c r="R165">
-        <v>1.13</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="S165">
         <v>4.05</v>
@@ -14856,7 +14233,7 @@
         <v>0.97</v>
       </c>
       <c r="U171">
-        <v>0.55</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="V171">
         <v>0.5</v>
@@ -15060,7 +14437,7 @@
         <v>2.06</v>
       </c>
       <c r="U174">
-        <v>0.55</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="V174">
         <v>1</v>
@@ -15128,7 +14505,7 @@
         <v>1.71</v>
       </c>
       <c r="U175">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="V175">
         <v>1</v>
@@ -15329,10 +14706,10 @@
         <v>2.33</v>
       </c>
       <c r="T178">
-        <v>2.03</v>
+        <v>2.0299999999999998</v>
       </c>
       <c r="U178">
-        <v>0.55</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="V178">
         <v>1</v>
@@ -15391,7 +14768,7 @@
         <v>2.33</v>
       </c>
       <c r="R179">
-        <v>2.03</v>
+        <v>2.0299999999999998</v>
       </c>
       <c r="S179">
         <v>2.06</v>
@@ -15400,7 +14777,7 @@
         <v>1.65</v>
       </c>
       <c r="U179">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="V179">
         <v>1</v>
@@ -15465,7 +14842,7 @@
         <v>5.01</v>
       </c>
       <c r="T180">
-        <v>1.14</v>
+        <v>1.1399999999999999</v>
       </c>
       <c r="U180">
         <v>0.64</v>
@@ -15536,7 +14913,7 @@
         <v>1.08</v>
       </c>
       <c r="U181">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="V181">
         <v>9999</v>
@@ -15601,7 +14978,7 @@
         <v>5.49</v>
       </c>
       <c r="T182">
-        <v>1.11</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="U182">
         <v>0.59</v>
@@ -15663,13 +15040,13 @@
         <v>5.49</v>
       </c>
       <c r="R183">
-        <v>1.11</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="S183">
         <v>5.3</v>
       </c>
       <c r="T183">
-        <v>1.11</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="U183">
         <v>0.62</v>
@@ -15808,7 +15185,7 @@
         <v>6.16</v>
       </c>
       <c r="U185">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="V185">
         <v>0.66</v>
@@ -16012,7 +15389,7 @@
         <v>7.12</v>
       </c>
       <c r="U188">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="V188">
         <v>1</v>
@@ -16133,13 +15510,13 @@
         <v>130</v>
       </c>
       <c r="Q190">
-        <v>4.4</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="R190">
         <v>0.88</v>
       </c>
       <c r="S190">
-        <v>4.35</v>
+        <v>4.3499999999999996</v>
       </c>
       <c r="T190">
         <v>0.92</v>
@@ -16207,7 +15584,7 @@
         <v>15.12</v>
       </c>
       <c r="S191">
-        <v>78.76</v>
+        <v>78.760000000000005</v>
       </c>
       <c r="T191">
         <v>16.66</v>
@@ -16269,7 +15646,7 @@
         <v>85</v>
       </c>
       <c r="Q192">
-        <v>39.27</v>
+        <v>39.270000000000003</v>
       </c>
       <c r="R192">
         <v>6.72</v>
@@ -16343,7 +15720,7 @@
         <v>5.94</v>
       </c>
       <c r="S193">
-        <v>38.8</v>
+        <v>38.799999999999997</v>
       </c>
       <c r="T193">
         <v>5.98</v>
@@ -16668,13 +16045,13 @@
         <v>4.18</v>
       </c>
       <c r="R198">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="S198">
         <v>4.07</v>
       </c>
       <c r="T198">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="U198">
         <v>0.53</v>
@@ -16736,7 +16113,7 @@
         <v>4.07</v>
       </c>
       <c r="R199">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="S199">
         <v>4</v>
@@ -16810,7 +16187,7 @@
         <v>3.94</v>
       </c>
       <c r="T200">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="U200">
         <v>0.66</v>
@@ -16872,7 +16249,7 @@
         <v>3.94</v>
       </c>
       <c r="R201">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="S201">
         <v>3.69</v>
@@ -16937,13 +16314,13 @@
         <v>48</v>
       </c>
       <c r="Q202">
-        <v>8.71</v>
+        <v>8.7100000000000009</v>
       </c>
       <c r="R202">
         <v>1.19</v>
       </c>
       <c r="S202">
-        <v>8.53</v>
+        <v>8.5299999999999994</v>
       </c>
       <c r="T202">
         <v>1.28</v>
@@ -17008,7 +16385,7 @@
         <v>8.6</v>
       </c>
       <c r="R203">
-        <v>1.13</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="S203">
         <v>8.48</v>
@@ -17419,7 +16796,7 @@
         <v>3.6</v>
       </c>
       <c r="S209">
-        <v>18.1</v>
+        <v>18.100000000000001</v>
       </c>
       <c r="T209">
         <v>4.2</v>
@@ -17481,7 +16858,7 @@
         <v>157</v>
       </c>
       <c r="Q210">
-        <v>18.1</v>
+        <v>18.100000000000001</v>
       </c>
       <c r="R210">
         <v>4.2</v>
@@ -17753,7 +17130,7 @@
         <v>162</v>
       </c>
       <c r="Q214">
-        <v>4.23</v>
+        <v>4.2300000000000004</v>
       </c>
       <c r="R214">
         <v>0.91</v>
@@ -17892,10 +17269,10 @@
         <v>4.18</v>
       </c>
       <c r="R216">
-        <v>1.15</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="S216">
-        <v>4.27</v>
+        <v>4.2699999999999996</v>
       </c>
       <c r="T216">
         <v>0.97</v>
@@ -18031,13 +17408,13 @@
         <v>1.34</v>
       </c>
       <c r="S218">
-        <v>4.73</v>
+        <v>4.7300000000000004</v>
       </c>
       <c r="T218">
         <v>1.31</v>
       </c>
       <c r="U218">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="V218">
         <v>0.5</v>
@@ -18093,7 +17470,7 @@
         <v>130</v>
       </c>
       <c r="Q219">
-        <v>4.73</v>
+        <v>4.7300000000000004</v>
       </c>
       <c r="R219">
         <v>1.31</v>
@@ -18161,7 +17538,7 @@
         <v>130</v>
       </c>
       <c r="Q220">
-        <v>4.77</v>
+        <v>4.7699999999999996</v>
       </c>
       <c r="R220">
         <v>1.34</v>
@@ -18241,7 +17618,7 @@
         <v>1.22</v>
       </c>
       <c r="U221">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="V221">
         <v>0.5</v>
@@ -18306,7 +17683,7 @@
         <v>5.01</v>
       </c>
       <c r="T222">
-        <v>1.16</v>
+        <v>1.1599999999999999</v>
       </c>
       <c r="U222">
         <v>0.62</v>
@@ -18439,13 +17816,13 @@
         <v>1.34</v>
       </c>
       <c r="S224">
-        <v>4.73</v>
+        <v>4.7300000000000004</v>
       </c>
       <c r="T224">
         <v>1.31</v>
       </c>
       <c r="U224">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="V224">
         <v>0.5</v>
@@ -18501,7 +17878,7 @@
         <v>130</v>
       </c>
       <c r="Q225">
-        <v>4.73</v>
+        <v>4.7300000000000004</v>
       </c>
       <c r="R225">
         <v>1.31</v>
@@ -18569,7 +17946,7 @@
         <v>130</v>
       </c>
       <c r="Q226">
-        <v>4.77</v>
+        <v>4.7699999999999996</v>
       </c>
       <c r="R226">
         <v>1.34</v>
@@ -18649,7 +18026,7 @@
         <v>1.22</v>
       </c>
       <c r="U227">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="V227">
         <v>0.5</v>
@@ -18714,7 +18091,7 @@
         <v>5.01</v>
       </c>
       <c r="T228">
-        <v>1.16</v>
+        <v>1.1599999999999999</v>
       </c>
       <c r="U228">
         <v>0.62</v>
@@ -18915,13 +18292,13 @@
         <v>1.41</v>
       </c>
       <c r="S231">
-        <v>4.9</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="T231">
         <v>1.27</v>
       </c>
       <c r="U231">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="V231">
         <v>1</v>
@@ -18977,13 +18354,13 @@
         <v>112</v>
       </c>
       <c r="Q232">
-        <v>4.9</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="R232">
         <v>1.27</v>
       </c>
       <c r="S232">
-        <v>4.9</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="T232">
         <v>1.25</v>
@@ -19122,7 +18499,7 @@
         <v>3.4</v>
       </c>
       <c r="T234">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="U234">
         <v>0.47</v>
@@ -19181,13 +18558,13 @@
         <v>57</v>
       </c>
       <c r="Q235">
-        <v>2.26</v>
+        <v>2.2599999999999998</v>
       </c>
       <c r="R235">
         <v>0.64</v>
       </c>
       <c r="S235">
-        <v>2.24</v>
+        <v>2.2400000000000002</v>
       </c>
       <c r="T235">
         <v>0.64</v>
@@ -19249,7 +18626,7 @@
         <v>57</v>
       </c>
       <c r="Q236">
-        <v>2.24</v>
+        <v>2.2400000000000002</v>
       </c>
       <c r="R236">
         <v>0.64</v>
@@ -19589,7 +18966,7 @@
         <v>187</v>
       </c>
       <c r="Q241">
-        <v>2.22</v>
+        <v>2.2200000000000002</v>
       </c>
       <c r="R241">
         <v>0.68</v>
@@ -19737,7 +19114,7 @@
         <v>0.53</v>
       </c>
       <c r="U243">
-        <v>0.55</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="V243">
         <v>1</v>
@@ -19997,7 +19374,7 @@
         <v>112</v>
       </c>
       <c r="Q247">
-        <v>19.83</v>
+        <v>19.829999999999998</v>
       </c>
       <c r="R247">
         <v>5.37</v>
@@ -20009,7 +19386,7 @@
         <v>5.43</v>
       </c>
       <c r="U247">
-        <v>0.568</v>
+        <v>0.56799999999999995</v>
       </c>
       <c r="V247">
         <v>1</v>
@@ -20071,7 +19448,7 @@
         <v>5.43</v>
       </c>
       <c r="S248">
-        <v>18.9</v>
+        <v>18.899999999999999</v>
       </c>
       <c r="T248">
         <v>5.27</v>
@@ -20133,7 +19510,7 @@
         <v>112</v>
       </c>
       <c r="Q249">
-        <v>18.9</v>
+        <v>18.899999999999999</v>
       </c>
       <c r="R249">
         <v>5.27</v>
@@ -20145,7 +19522,7 @@
         <v>5.27</v>
       </c>
       <c r="U249">
-        <v>0.593</v>
+        <v>0.59299999999999997</v>
       </c>
       <c r="V249">
         <v>1</v>
@@ -20662,7 +20039,7 @@
         <v>7.69</v>
       </c>
       <c r="R257">
-        <v>2.05</v>
+        <v>2.0499999999999998</v>
       </c>
       <c r="S257">
         <v>7.74</v>
@@ -20792,7 +20169,7 @@
         <v>7.61</v>
       </c>
       <c r="T259">
-        <v>2.43</v>
+        <v>2.4300000000000002</v>
       </c>
       <c r="U259">
         <v>9999</v>
@@ -20848,7 +20225,7 @@
         <v>7.61</v>
       </c>
       <c r="R260">
-        <v>2.43</v>
+        <v>2.4300000000000002</v>
       </c>
       <c r="S260">
         <v>8.06</v>
@@ -21031,7 +20408,7 @@
         <v>129</v>
       </c>
       <c r="Q263">
-        <v>8.53</v>
+        <v>8.5299999999999994</v>
       </c>
       <c r="R263">
         <v>1.84</v>
@@ -21040,7 +20417,7 @@
         <v>8.16</v>
       </c>
       <c r="T263">
-        <v>2.32</v>
+        <v>2.3199999999999998</v>
       </c>
       <c r="U263">
         <v>9999</v>
@@ -21096,7 +20473,7 @@
         <v>8.16</v>
       </c>
       <c r="R264">
-        <v>2.32</v>
+        <v>2.3199999999999998</v>
       </c>
       <c r="S264">
         <v>7.9</v>
@@ -21161,16 +20538,16 @@
         <v>85</v>
       </c>
       <c r="Q265">
-        <v>5.11</v>
+        <v>5.1100000000000003</v>
       </c>
       <c r="R265">
         <v>1.07</v>
       </c>
       <c r="S265">
-        <v>5.11</v>
+        <v>5.1100000000000003</v>
       </c>
       <c r="T265">
-        <v>1.15</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="U265">
         <v>0.65</v>
@@ -21229,10 +20606,10 @@
         <v>85</v>
       </c>
       <c r="Q266">
-        <v>5.11</v>
+        <v>5.1100000000000003</v>
       </c>
       <c r="R266">
-        <v>1.15</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="S266">
         <v>5.26</v>
@@ -21306,7 +20683,7 @@
         <v>5.3</v>
       </c>
       <c r="T267">
-        <v>1.15</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="U267">
         <v>0.65</v>
@@ -21492,7 +20869,7 @@
         <v>3.8</v>
       </c>
       <c r="R270">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="S270">
         <v>3.83</v>
@@ -21566,7 +20943,7 @@
         <v>3.94</v>
       </c>
       <c r="T271">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="U271">
         <v>0.21</v>
@@ -21835,7 +21212,7 @@
         <v>0.89</v>
       </c>
       <c r="S275">
-        <v>2.49</v>
+        <v>2.4900000000000002</v>
       </c>
       <c r="T275">
         <v>0.89</v>
@@ -22104,7 +21481,7 @@
         <v>3.47</v>
       </c>
       <c r="T279">
-        <v>1.13</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="U279">
         <v>0.43</v>
@@ -22166,7 +21543,7 @@
         <v>3.47</v>
       </c>
       <c r="R280">
-        <v>1.13</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="S280">
         <v>3.56</v>
@@ -22379,7 +21756,7 @@
         <v>7.92</v>
       </c>
       <c r="U283">
-        <v>0.785</v>
+        <v>0.78500000000000003</v>
       </c>
       <c r="V283">
         <v>1</v>
@@ -22991,7 +22368,7 @@
         <v>0.74</v>
       </c>
       <c r="U292">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="V292">
         <v>1</v>
@@ -23124,7 +22501,7 @@
         <v>3.85</v>
       </c>
       <c r="T294">
-        <v>1.09</v>
+        <v>1.0900000000000001</v>
       </c>
       <c r="U294">
         <v>0.54</v>
@@ -23331,7 +22708,7 @@
         <v>3.08</v>
       </c>
       <c r="U297">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="V297">
         <v>0.5</v>
@@ -23399,7 +22776,7 @@
         <v>2.91</v>
       </c>
       <c r="U298">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="V298">
         <v>0.5</v>
@@ -23671,7 +23048,7 @@
         <v>0.77</v>
       </c>
       <c r="U302">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="V302">
         <v>0.5</v>
@@ -24141,7 +23518,7 @@
         <v>0.78</v>
       </c>
       <c r="S309">
-        <v>2.51</v>
+        <v>2.5099999999999998</v>
       </c>
       <c r="T309">
         <v>0.74</v>
@@ -24203,7 +23580,7 @@
         <v>118</v>
       </c>
       <c r="Q310">
-        <v>2.51</v>
+        <v>2.5099999999999998</v>
       </c>
       <c r="R310">
         <v>0.74</v>
@@ -24759,7 +24136,7 @@
         <v>0.72</v>
       </c>
       <c r="U318">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="V318">
         <v>0.5</v>
@@ -25028,7 +24405,7 @@
         <v>5.69</v>
       </c>
       <c r="T322">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="U322">
         <v>9999</v>
@@ -25096,7 +24473,7 @@
         <v>2.54</v>
       </c>
       <c r="T323">
-        <v>1.09</v>
+        <v>1.0900000000000001</v>
       </c>
       <c r="U323">
         <v>9999</v>
@@ -25158,7 +24535,7 @@
         <v>2.54</v>
       </c>
       <c r="R324">
-        <v>1.09</v>
+        <v>1.0900000000000001</v>
       </c>
       <c r="S324">
         <v>2.38</v>
@@ -25300,7 +24677,7 @@
         <v>2.57</v>
       </c>
       <c r="T326">
-        <v>1.13</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="U326">
         <v>9999</v>
@@ -25977,7 +25354,7 @@
         <v>0.71</v>
       </c>
       <c r="S336">
-        <v>2.45</v>
+        <v>2.4500000000000002</v>
       </c>
       <c r="T336">
         <v>0.41</v>
@@ -26048,7 +25425,7 @@
         <v>4.91</v>
       </c>
       <c r="T337">
-        <v>1.11</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="U337">
         <v>0.54</v>
@@ -26110,7 +25487,7 @@
         <v>4.62</v>
       </c>
       <c r="R338">
-        <v>1.13</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="S338">
         <v>4.54</v>
@@ -26385,7 +25762,7 @@
         <v>0.73</v>
       </c>
       <c r="S342">
-        <v>2.55</v>
+        <v>2.5499999999999998</v>
       </c>
       <c r="T342">
         <v>0.71</v>
@@ -26651,13 +26028,13 @@
         <v>222</v>
       </c>
       <c r="Q346">
-        <v>18.56</v>
+        <v>18.559999999999999</v>
       </c>
       <c r="R346">
         <v>4.79</v>
       </c>
       <c r="S346">
-        <v>17.51</v>
+        <v>17.510000000000002</v>
       </c>
       <c r="T346">
         <v>5.2</v>
@@ -26719,7 +26096,7 @@
         <v>130</v>
       </c>
       <c r="Q347">
-        <v>4.4</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="R347">
         <v>1.21</v>
@@ -26728,7 +26105,7 @@
         <v>4.09</v>
       </c>
       <c r="T347">
-        <v>1.14</v>
+        <v>1.1399999999999999</v>
       </c>
       <c r="U347">
         <v>9999</v>
@@ -26790,7 +26167,7 @@
         <v>4.09</v>
       </c>
       <c r="R348">
-        <v>1.14</v>
+        <v>1.1399999999999999</v>
       </c>
       <c r="S348">
         <v>4.05</v>
@@ -27269,7 +26646,7 @@
         <v>1.26</v>
       </c>
       <c r="S355">
-        <v>4.81</v>
+        <v>4.8099999999999996</v>
       </c>
       <c r="T355">
         <v>1.34</v>
@@ -27337,7 +26714,7 @@
         <v>1.31</v>
       </c>
       <c r="S356">
-        <v>4.94</v>
+        <v>4.9400000000000004</v>
       </c>
       <c r="T356">
         <v>1.06</v>
@@ -27408,7 +26785,7 @@
         <v>5.31</v>
       </c>
       <c r="T357">
-        <v>1.14</v>
+        <v>1.1399999999999999</v>
       </c>
       <c r="U357">
         <v>0.37</v>
@@ -27795,7 +27172,7 @@
         <v>7.2</v>
       </c>
       <c r="S363">
-        <v>33.3</v>
+        <v>33.299999999999997</v>
       </c>
       <c r="T363">
         <v>6.6</v>
@@ -27857,13 +27234,13 @@
         <v>85</v>
       </c>
       <c r="Q364">
-        <v>33.3</v>
+        <v>33.299999999999997</v>
       </c>
       <c r="R364">
         <v>6.6</v>
       </c>
       <c r="S364">
-        <v>33.7</v>
+        <v>33.700000000000003</v>
       </c>
       <c r="T364">
         <v>6.1</v>
@@ -27925,7 +27302,7 @@
         <v>85</v>
       </c>
       <c r="Q365">
-        <v>33.7</v>
+        <v>33.700000000000003</v>
       </c>
       <c r="R365">
         <v>6.1</v>
@@ -28883,10 +28260,10 @@
         <v>1.28</v>
       </c>
       <c r="S379">
-        <v>4.27</v>
+        <v>4.2699999999999996</v>
       </c>
       <c r="T379">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="U379">
         <v>0.31</v>
@@ -29480,7 +28857,7 @@
         <v>14.59</v>
       </c>
       <c r="T388">
-        <v>4.81</v>
+        <v>4.8099999999999996</v>
       </c>
       <c r="U388">
         <v>9999</v>
@@ -29814,13 +29191,13 @@
         <v>5.38</v>
       </c>
       <c r="R393">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="S393">
         <v>5.36</v>
       </c>
       <c r="T393">
-        <v>1.09</v>
+        <v>1.0900000000000001</v>
       </c>
       <c r="U393">
         <v>0.47</v>
@@ -29888,7 +29265,7 @@
         <v>30.93</v>
       </c>
       <c r="T394">
-        <v>8.79</v>
+        <v>8.7899999999999991</v>
       </c>
       <c r="U394">
         <v>9999</v>
@@ -29950,7 +29327,7 @@
         <v>30.93</v>
       </c>
       <c r="R395">
-        <v>8.79</v>
+        <v>8.7899999999999991</v>
       </c>
       <c r="S395">
         <v>31.1</v>
@@ -30024,7 +29401,7 @@
         <v>31.62</v>
       </c>
       <c r="T396">
-        <v>8.87</v>
+        <v>8.8699999999999992</v>
       </c>
       <c r="U396">
         <v>9999</v>
@@ -30086,7 +29463,7 @@
         <v>31.62</v>
       </c>
       <c r="R397">
-        <v>8.87</v>
+        <v>8.8699999999999992</v>
       </c>
       <c r="S397">
         <v>31.68</v>
@@ -30228,7 +29605,7 @@
         <v>19.84</v>
       </c>
       <c r="T399">
-        <v>9.03</v>
+        <v>9.0299999999999994</v>
       </c>
       <c r="U399">
         <v>9999</v>
@@ -30296,7 +29673,7 @@
         <v>22.06</v>
       </c>
       <c r="T400">
-        <v>8.53</v>
+        <v>8.5299999999999994</v>
       </c>
       <c r="U400">
         <v>9999</v>
@@ -30364,7 +29741,7 @@
         <v>22.24</v>
       </c>
       <c r="T401">
-        <v>8.55</v>
+        <v>8.5500000000000007</v>
       </c>
       <c r="U401">
         <v>9999</v>
@@ -31180,7 +30557,7 @@
         <v>3.71</v>
       </c>
       <c r="T413">
-        <v>1.09</v>
+        <v>1.0900000000000001</v>
       </c>
       <c r="U413">
         <v>9999</v>
@@ -31307,7 +30684,7 @@
         <v>112</v>
       </c>
       <c r="Q415">
-        <v>4.15</v>
+        <v>4.1500000000000004</v>
       </c>
       <c r="R415">
         <v>0.77</v>
@@ -31381,7 +30758,7 @@
         <v>0.8</v>
       </c>
       <c r="S416">
-        <v>4.14</v>
+        <v>4.1399999999999997</v>
       </c>
       <c r="T416">
         <v>0.81</v>
@@ -31446,16 +30823,16 @@
         <v>4.22</v>
       </c>
       <c r="R417">
-        <v>1.14</v>
+        <v>1.1399999999999999</v>
       </c>
       <c r="S417">
-        <v>4.27</v>
+        <v>4.2699999999999996</v>
       </c>
       <c r="T417">
-        <v>1.11</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="U417">
-        <v>0.56</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="V417">
         <v>1</v>
@@ -31511,7 +30888,7 @@
         <v>162</v>
       </c>
       <c r="Q418">
-        <v>4.15</v>
+        <v>4.1500000000000004</v>
       </c>
       <c r="R418">
         <v>1.01</v>
@@ -31653,13 +31030,13 @@
         <v>1.08</v>
       </c>
       <c r="S420">
-        <v>4.39</v>
+        <v>4.3899999999999997</v>
       </c>
       <c r="T420">
-        <v>1.09</v>
+        <v>1.0900000000000001</v>
       </c>
       <c r="U420">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="V420">
         <v>0.5</v>
@@ -31715,19 +31092,19 @@
         <v>162</v>
       </c>
       <c r="Q421">
-        <v>4.39</v>
+        <v>4.3899999999999997</v>
       </c>
       <c r="R421">
-        <v>1.09</v>
+        <v>1.0900000000000001</v>
       </c>
       <c r="S421">
-        <v>4.44</v>
+        <v>4.4400000000000004</v>
       </c>
       <c r="T421">
-        <v>1.15</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="U421">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="V421">
         <v>0.5</v>
@@ -31851,7 +31228,7 @@
         <v>111</v>
       </c>
       <c r="Q423">
-        <v>4.73</v>
+        <v>4.7300000000000004</v>
       </c>
       <c r="R423">
         <v>0.81</v>
@@ -31919,13 +31296,13 @@
         <v>111</v>
       </c>
       <c r="Q424">
-        <v>4.69</v>
+        <v>4.6900000000000004</v>
       </c>
       <c r="R424">
         <v>0.78</v>
       </c>
       <c r="S424">
-        <v>4.56</v>
+        <v>4.5599999999999996</v>
       </c>
       <c r="T424">
         <v>0.78</v>
@@ -32652,10 +32029,10 @@
         <v>1.02</v>
       </c>
       <c r="S435">
-        <v>2.47</v>
+        <v>2.4700000000000002</v>
       </c>
       <c r="T435">
-        <v>1.11</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="U435">
         <v>9999</v>
@@ -32711,10 +32088,10 @@
         <v>56</v>
       </c>
       <c r="Q436">
-        <v>2.47</v>
+        <v>2.4700000000000002</v>
       </c>
       <c r="R436">
-        <v>1.11</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="S436">
         <v>2.36</v>
@@ -32782,7 +32159,7 @@
         <v>1.02</v>
       </c>
       <c r="S437">
-        <v>2.45</v>
+        <v>2.4500000000000002</v>
       </c>
       <c r="T437">
         <v>1.17</v>
@@ -32841,7 +32218,7 @@
         <v>56</v>
       </c>
       <c r="Q438">
-        <v>2.45</v>
+        <v>2.4500000000000002</v>
       </c>
       <c r="R438">
         <v>1.17</v>
@@ -32906,7 +32283,7 @@
         <v>56</v>
       </c>
       <c r="Q439">
-        <v>2.47</v>
+        <v>2.4700000000000002</v>
       </c>
       <c r="R439">
         <v>0.93</v>
@@ -33107,7 +32484,7 @@
         <v>84</v>
       </c>
       <c r="Q442">
-        <v>4.81</v>
+        <v>4.8099999999999996</v>
       </c>
       <c r="R442">
         <v>1.33</v>
@@ -33320,7 +32697,7 @@
         <v>5.14</v>
       </c>
       <c r="T445">
-        <v>1.12</v>
+        <v>1.1200000000000001</v>
       </c>
       <c r="U445">
         <v>9999</v>
@@ -34248,16 +33625,16 @@
         <v>33</v>
       </c>
       <c r="Q459">
-        <v>4.06</v>
+        <v>4.0599999999999996</v>
       </c>
       <c r="R459">
-        <v>1.12</v>
+        <v>1.1200000000000001</v>
       </c>
       <c r="S459">
-        <v>4.06</v>
+        <v>4.0599999999999996</v>
       </c>
       <c r="T459">
-        <v>1.13</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="U459">
         <v>0.38</v>
@@ -34609,6 +33986,5 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>